<commit_message>
docs: harden published teaching workbooks
</commit_message>
<xml_diff>
--- a/docs/tutorial-assets/workbooks/01_PyroApp_Getting_Started_Ca-Zn-O.xlsx
+++ b/docs/tutorial-assets/workbooks/01_PyroApp_Getting_Started_Ca-Zn-O.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\_WORK\Code\Rust\pyroapp-docs\docs\tutorial-assets\workbooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{428333E2-A185-4A23-8571-1E30F0E42820}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90D475CB-6AB7-4BD1-BF4B-CBA66AF118F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-51720" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,9 +41,10 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="2">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
   </metadataTypes>
   <futureMetadata name="XLDAPR" count="1">
     <bk>
@@ -54,11 +55,35 @@
       </extLst>
     </bk>
   </futureMetadata>
+  <futureMetadata name="XLRICHVALUE" count="2">
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="0"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="1"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
   <cellMetadata count="1">
     <bk>
       <rc t="1" v="0"/>
     </bk>
   </cellMetadata>
+  <valueMetadata count="2">
+    <bk>
+      <rc t="2" v="0"/>
+    </bk>
+    <bk>
+      <rc t="2" v="1"/>
+    </bk>
+  </valueMetadata>
 </metadata>
 </file>
 
@@ -592,7 +617,7 @@
           <c:smooth val="1"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-62D4-48E2-99D6-73C9DF7EA8E9}"/>
+              <c16:uniqueId val="{00000000-CBFA-4968-B318-B31CD086E189}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -697,7 +722,7 @@
           <c:smooth val="1"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-62D4-48E2-99D6-73C9DF7EA8E9}"/>
+              <c16:uniqueId val="{00000001-CBFA-4968-B318-B31CD086E189}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -802,7 +827,7 @@
           <c:smooth val="1"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-62D4-48E2-99D6-73C9DF7EA8E9}"/>
+              <c16:uniqueId val="{00000002-CBFA-4968-B318-B31CD086E189}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1040,7 +1065,7 @@
           <c:smooth val="1"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-B3A7-47C5-86D4-7F8C88A90A0D}"/>
+              <c16:uniqueId val="{00000000-31E1-4FA6-8A30-45BE9D5B19CC}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1151,7 +1176,7 @@
           <c:smooth val="1"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-B3A7-47C5-86D4-7F8C88A90A0D}"/>
+              <c16:uniqueId val="{00000001-31E1-4FA6-8A30-45BE9D5B19CC}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1262,7 +1287,7 @@
           <c:smooth val="1"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-B3A7-47C5-86D4-7F8C88A90A0D}"/>
+              <c16:uniqueId val="{00000002-31E1-4FA6-8A30-45BE9D5B19CC}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1433,6 +1458,74 @@
     <xdr:clientData/>
   </xdr:oneCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
+<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
+  <global>
+    <keyFlags>
+      <key name="_Self">
+        <flag name="ExcludeFromFile" value="1"/>
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_DisplayString">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Flags">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Format">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_SubLabel">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Attribution">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Icon">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Display">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_CanonicalPropertyNames">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_ClassificationId">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+    </keyFlags>
+  </global>
+</rvTypesInfo>
+</file>
+
+<file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="2">
+  <rv s="0">
+    <v>1</v>
+    <v>8</v>
+    <v>10</v>
+    <v>1</v>
+  </rv>
+  <rv s="0">
+    <v>0</v>
+    <v>8</v>
+    <v>17</v>
+    <v>1</v>
+  </rv>
+</rvData>
+</file>
+
+<file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
+<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+  <s t="_error">
+    <k n="colOffset" t="i"/>
+    <k n="errorType" t="i"/>
+    <k n="rwOffset" t="i"/>
+    <k n="subType" t="i"/>
+  </s>
+</rvStructures>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1869,12 +1962,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="19.90625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="52.08984375" bestFit="1" customWidth="1"/>
-    <col min="3" max="16" width="18" customWidth="1"/>
+    <col min="2" max="2" width="26.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="2.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="16" width="18" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="23.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
@@ -1895,8 +1989,8 @@
       <c r="A5" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="1">
-        <f>_xll.XLL_CA_VERSION()</f>
+      <c r="B5" s="1" cm="1">
+        <f t="array" ref="B5">_xll.XLL_CA_VERSION()</f>
         <v>714</v>
       </c>
     </row>
@@ -1904,8 +1998,8 @@
       <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="1" t="b">
-        <f>_xll.XLL_CA_ISLITE()</f>
+      <c r="B6" s="1" t="b" cm="1">
+        <f t="array" ref="B6">_xll.XLL_CA_ISLITE()</f>
         <v>0</v>
       </c>
     </row>
@@ -1913,8 +2007,8 @@
       <c r="A7" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="1" t="str">
-        <f>_xll.XLL_CA_USER_ID()</f>
+      <c r="B7" s="1" t="str" cm="1">
+        <f t="array" ref="B7">_xll.XLL_CA_USER_ID()</f>
         <v>0040</v>
       </c>
     </row>
@@ -1922,8 +2016,8 @@
       <c r="A8" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="1" t="str">
-        <f>_xll.XLL_CA_LICENSE_HOLDER_NAME()</f>
+      <c r="B8" s="1" t="str" cm="1">
+        <f t="array" ref="B8">_xll.XLL_CA_LICENSE_HOLDER_NAME()</f>
         <v>University</v>
       </c>
     </row>
@@ -1931,8 +2025,8 @@
       <c r="A9" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B9" s="1" t="str">
-        <f>_xll.XLL_CA_PROGRAM_ID()</f>
+      <c r="B9" s="1" t="str" cm="1">
+        <f t="array" ref="B9">_xll.XLL_CA_PROGRAM_ID()</f>
         <v>CAFU</v>
       </c>
     </row>
@@ -1940,27 +2034,46 @@
       <c r="A10" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B10" s="1" t="str">
-        <f>_xll.XLL_CA_DIMENSIONS_MAX()</f>
-        <v>number_phase_constituents</v>
+      <c r="B10" s="1" t="e" cm="1" vm="1">
+        <f t="array" aca="1" ref="B10" ca="1">_xll.XLL_CA_DIMENSIONS_MAX()</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="1" t="str">
-        <f>_xll.XLL_CA_CHEMAPPDLLS()</f>
-        <v>C:\Program Files\PYROAPP\x64\ChemApp\chemapp_00.dll</v>
+      <c r="B11" s="1" t="e" cm="1" vm="2">
+        <f t="array" aca="1" ref="B11" ca="1">_xll.XLL_CA_CHEMAPPDLLS()</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B12" s="1" t="str">
-        <f>_xll.XLL_CA_DIMENSIONS(Start!$B$10)</f>
+      <c r="B12" s="1" t="str" cm="1">
+        <f t="array" ref="B12:C14">_xll.XLL_CA_DIMENSIONS(Start!$B$10)</f>
         <v>number_system_components</v>
+      </c>
+      <c r="C12">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B13" t="str">
+        <v>number_phases</v>
+      </c>
+      <c r="C13">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B14" t="str">
+        <v>number_phase_constituents</v>
+      </c>
+      <c r="C14">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -2171,8 +2284,8 @@
       <c r="A28" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B28" s="1">
-        <f>_xll.XLL_CA_GET_COMPONENT_WEIGHTS(Start!$B$10,"Zn")</f>
+      <c r="B28" s="1" cm="1">
+        <f t="array" ref="B28">_xll.XLL_CA_GET_COMPONENT_WEIGHTS(Start!$B$10,"Zn")</f>
         <v>65.38</v>
       </c>
     </row>
@@ -2180,8 +2293,8 @@
       <c r="A29" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B29" s="1">
-        <f>_xll.XLL_CA_GET_COMPONENT_WEIGHTS(Start!$B$10,"Ca")</f>
+      <c r="B29" s="1" cm="1">
+        <f t="array" ref="B29">_xll.XLL_CA_GET_COMPONENT_WEIGHTS(Start!$B$10,"Ca")</f>
         <v>40.078000000000003</v>
       </c>
     </row>
@@ -2189,8 +2302,8 @@
       <c r="A30" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B30" s="1">
-        <f>_xll.XLL_CA_GET_COMPOUND_H298(Start!$B$10,"ZnO(s)")</f>
+      <c r="B30" s="1" cm="1">
+        <f t="array" ref="B30">_xll.XLL_CA_GET_COMPOUND_H298(Start!$B$10,"ZnO(s)")</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>